<commit_message>
feat: add default institutional report structure, stop-slop narrative, and dual .agents support
</commit_message>
<xml_diff>
--- a/examples/sample-report/tables.xlsx
+++ b/examples/sample-report/tables.xlsx
@@ -11,17 +11,88 @@
     <sheet name="Table2" sheetId="2" r:id="rId2"/>
     <sheet name="Table3" sheetId="3" r:id="rId3"/>
     <sheet name="Table4" sheetId="4" r:id="rId4"/>
+    <sheet name="Table5" sheetId="5" r:id="rId5"/>
+    <sheet name="Table6" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="103">
   <si>
     <t>Değişken</t>
   </si>
   <si>
+    <t>Veri Türü</t>
+  </si>
+  <si>
+    <t>Geçerli N</t>
+  </si>
+  <si>
+    <t>Kayıp Oranı</t>
+  </si>
+  <si>
+    <t>Tekil Değer</t>
+  </si>
+  <si>
+    <t>Katılımcı No</t>
+  </si>
+  <si>
+    <t>Yaş</t>
+  </si>
+  <si>
+    <t>Cinsiyet</t>
+  </si>
+  <si>
+    <t>Eğitim Düzeyi</t>
+  </si>
+  <si>
+    <t>İş Tatmini</t>
+  </si>
+  <si>
+    <t>Tükenmişlik</t>
+  </si>
+  <si>
+    <t>Özyeterlik</t>
+  </si>
+  <si>
+    <t>Sürekli (Sayısal)</t>
+  </si>
+  <si>
+    <t>Kategorik</t>
+  </si>
+  <si>
+    <t>300</t>
+  </si>
+  <si>
+    <t>285</t>
+  </si>
+  <si>
+    <t>%0,0</t>
+  </si>
+  <si>
+    <t>%5,0</t>
+  </si>
+  <si>
+    <t>47</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>37</t>
+  </si>
+  <si>
+    <t>39</t>
+  </si>
+  <si>
+    <t>35</t>
+  </si>
+  <si>
     <t>n</t>
   </si>
   <si>
@@ -37,24 +108,6 @@
     <t>Basıklık</t>
   </si>
   <si>
-    <t>Yaş</t>
-  </si>
-  <si>
-    <t>İş Tatmini</t>
-  </si>
-  <si>
-    <t>Tükenmişlik</t>
-  </si>
-  <si>
-    <t>Özyeterlik</t>
-  </si>
-  <si>
-    <t>300</t>
-  </si>
-  <si>
-    <t>285</t>
-  </si>
-  <si>
     <t>41,76</t>
   </si>
   <si>
@@ -103,12 +156,6 @@
     <t>1</t>
   </si>
   <si>
-    <t>2</t>
-  </si>
-  <si>
-    <t>3</t>
-  </si>
-  <si>
     <t>1. Yaş</t>
   </si>
   <si>
@@ -242,6 +289,45 @@
   </si>
   <si>
     <t>1,1</t>
+  </si>
+  <si>
+    <t>Min</t>
+  </si>
+  <si>
+    <t>Maks</t>
+  </si>
+  <si>
+    <t>1,00</t>
+  </si>
+  <si>
+    <t>18,00</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>1,60</t>
+  </si>
+  <si>
+    <t>300,00</t>
+  </si>
+  <si>
+    <t>64,00</t>
+  </si>
+  <si>
+    <t>4,80</t>
+  </si>
+  <si>
+    <t>5,00</t>
+  </si>
+  <si>
+    <t>5,20</t>
+  </si>
+  <si>
+    <t>150,50</t>
+  </si>
+  <si>
+    <t>86,75</t>
   </si>
 </sst>
 </file>
@@ -573,10 +659,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:5">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -592,88 +678,124 @@
       <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" spans="1:6">
-      <c r="A2" t="s">
-        <v>6</v>
-      </c>
       <c r="B2" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C2" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D2" t="s">
         <v>16</v>
       </c>
       <c r="E2" t="s">
-        <v>19</v>
-      </c>
-      <c r="F2" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5">
       <c r="A3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D3" t="s">
+        <v>16</v>
+      </c>
+      <c r="E3" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5">
+      <c r="A4" t="s">
         <v>7</v>
       </c>
-      <c r="B3" t="s">
-        <v>10</v>
-      </c>
-      <c r="C3" t="s">
+      <c r="B4" t="s">
         <v>13</v>
-      </c>
-      <c r="D3" t="s">
-        <v>17</v>
-      </c>
-      <c r="E3" t="s">
-        <v>20</v>
-      </c>
-      <c r="F3" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6">
-      <c r="A4" t="s">
-        <v>8</v>
-      </c>
-      <c r="B4" t="s">
-        <v>11</v>
       </c>
       <c r="C4" t="s">
         <v>14</v>
       </c>
       <c r="D4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E4" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5">
+      <c r="A5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D5" t="s">
+        <v>16</v>
+      </c>
+      <c r="E5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5">
+      <c r="A6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C6" t="s">
+        <v>14</v>
+      </c>
+      <c r="D6" t="s">
+        <v>16</v>
+      </c>
+      <c r="E6" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5">
+      <c r="A7" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7" t="s">
+        <v>12</v>
+      </c>
+      <c r="C7" t="s">
+        <v>15</v>
+      </c>
+      <c r="D7" t="s">
         <v>17</v>
       </c>
-      <c r="E4" t="s">
-        <v>21</v>
-      </c>
-      <c r="F4" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6">
-      <c r="A5" t="s">
-        <v>9</v>
-      </c>
-      <c r="B5" t="s">
-        <v>10</v>
-      </c>
-      <c r="C5" t="s">
-        <v>15</v>
-      </c>
-      <c r="D5" t="s">
-        <v>18</v>
-      </c>
-      <c r="E5" t="s">
+      <c r="E7" t="s">
         <v>22</v>
       </c>
-      <c r="F5" t="s">
-        <v>26</v>
+    </row>
+    <row r="8" spans="1:5">
+      <c r="A8" t="s">
+        <v>11</v>
+      </c>
+      <c r="B8" t="s">
+        <v>12</v>
+      </c>
+      <c r="C8" t="s">
+        <v>14</v>
+      </c>
+      <c r="D8" t="s">
+        <v>16</v>
+      </c>
+      <c r="E8" t="s">
+        <v>23</v>
       </c>
     </row>
   </sheetData>
@@ -683,59 +805,107 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:6">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C1" t="s">
+        <v>25</v>
+      </c>
+      <c r="D1" t="s">
+        <v>26</v>
+      </c>
+      <c r="E1" t="s">
         <v>27</v>
       </c>
-      <c r="C1" t="s">
+      <c r="F1" t="s">
         <v>28</v>
       </c>
-      <c r="D1" t="s">
+    </row>
+    <row r="2" spans="1:6">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C2" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="2" spans="1:4">
-      <c r="A2" t="s">
+      <c r="D2" t="s">
+        <v>33</v>
+      </c>
+      <c r="E2" t="s">
+        <v>36</v>
+      </c>
+      <c r="F2" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6">
+      <c r="A3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C3" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="3" spans="1:4">
-      <c r="A3" t="s">
+      <c r="D3" t="s">
+        <v>34</v>
+      </c>
+      <c r="E3" t="s">
+        <v>37</v>
+      </c>
+      <c r="F3" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6">
+      <c r="A4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C4" t="s">
         <v>31</v>
       </c>
-      <c r="B3" t="s">
+      <c r="D4" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="4" spans="1:4">
-      <c r="A4" t="s">
+      <c r="E4" t="s">
+        <v>38</v>
+      </c>
+      <c r="F4" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6">
+      <c r="A5" t="s">
+        <v>11</v>
+      </c>
+      <c r="B5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C5" t="s">
         <v>32</v>
       </c>
-      <c r="B4" t="s">
+      <c r="D5" t="s">
         <v>35</v>
       </c>
-      <c r="C4" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4">
-      <c r="A5" t="s">
-        <v>33</v>
-      </c>
-      <c r="B5" t="s">
-        <v>36</v>
-      </c>
-      <c r="C5" t="s">
-        <v>38</v>
-      </c>
-      <c r="D5" t="s">
+      <c r="E5" t="s">
         <v>39</v>
+      </c>
+      <c r="F5" t="s">
+        <v>43</v>
       </c>
     </row>
   </sheetData>
@@ -745,49 +915,59 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" t="s">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>1</v>
+        <v>44</v>
       </c>
       <c r="C1" t="s">
-        <v>2</v>
+        <v>19</v>
       </c>
       <c r="D1" t="s">
-        <v>3</v>
+        <v>20</v>
       </c>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" t="s">
-        <v>41</v>
-      </c>
-      <c r="B2" t="s">
-        <v>43</v>
-      </c>
-      <c r="C2" t="s">
         <v>45</v>
-      </c>
-      <c r="D2" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="B3" t="s">
-        <v>44</v>
-      </c>
-      <c r="C3" t="s">
-        <v>46</v>
-      </c>
-      <c r="D3" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="A4" t="s">
+        <v>47</v>
+      </c>
+      <c r="B4" t="s">
+        <v>50</v>
+      </c>
+      <c r="C4" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
+      <c r="A5" t="s">
         <v>48</v>
+      </c>
+      <c r="B5" t="s">
+        <v>51</v>
+      </c>
+      <c r="C5" t="s">
+        <v>53</v>
+      </c>
+      <c r="D5" t="s">
+        <v>54</v>
       </c>
     </row>
   </sheetData>
@@ -797,53 +977,105 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:D3"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:4">
+      <c r="A1" t="s">
+        <v>55</v>
+      </c>
+      <c r="B1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C1" t="s">
+        <v>25</v>
+      </c>
+      <c r="D1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B2" t="s">
+        <v>58</v>
+      </c>
+      <c r="C2" t="s">
+        <v>60</v>
+      </c>
+      <c r="D2" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
+      <c r="A3" t="s">
+        <v>57</v>
+      </c>
+      <c r="B3" t="s">
+        <v>59</v>
+      </c>
+      <c r="C3" t="s">
+        <v>61</v>
+      </c>
+      <c r="D3" t="s">
+        <v>63</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:G5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:7">
       <c r="A1" t="s">
-        <v>49</v>
+        <v>64</v>
       </c>
       <c r="B1" t="s">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="C1" t="s">
-        <v>51</v>
+        <v>66</v>
       </c>
       <c r="D1" t="s">
-        <v>52</v>
+        <v>67</v>
       </c>
       <c r="E1" t="s">
-        <v>53</v>
+        <v>68</v>
       </c>
       <c r="F1" t="s">
-        <v>54</v>
+        <v>69</v>
       </c>
       <c r="G1" t="s">
-        <v>55</v>
+        <v>70</v>
       </c>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" t="s">
-        <v>56</v>
+        <v>71</v>
       </c>
       <c r="B2" t="s">
-        <v>57</v>
+        <v>72</v>
       </c>
       <c r="C2" t="s">
-        <v>61</v>
+        <v>76</v>
       </c>
       <c r="D2" t="s">
-        <v>64</v>
+        <v>79</v>
       </c>
       <c r="E2" t="s">
-        <v>68</v>
+        <v>83</v>
       </c>
       <c r="F2" t="s">
-        <v>72</v>
+        <v>87</v>
       </c>
       <c r="G2" t="s">
-        <v>64</v>
+        <v>79</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -851,71 +1083,241 @@
         <v>6</v>
       </c>
       <c r="B3" t="s">
-        <v>58</v>
+        <v>73</v>
       </c>
       <c r="C3" t="s">
-        <v>58</v>
+        <v>73</v>
       </c>
       <c r="D3" t="s">
-        <v>65</v>
+        <v>80</v>
       </c>
       <c r="E3" t="s">
-        <v>69</v>
+        <v>84</v>
       </c>
       <c r="F3">
         <f> ,670</f>
         <v>0</v>
       </c>
       <c r="G3" t="s">
-        <v>73</v>
+        <v>88</v>
       </c>
     </row>
     <row r="4" spans="1:7">
       <c r="A4" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B4" t="s">
-        <v>59</v>
+        <v>74</v>
       </c>
       <c r="C4" t="s">
-        <v>62</v>
+        <v>77</v>
       </c>
       <c r="D4" t="s">
-        <v>66</v>
+        <v>81</v>
       </c>
       <c r="E4" t="s">
-        <v>70</v>
+        <v>85</v>
       </c>
       <c r="F4">
         <f> ,129</f>
         <v>0</v>
       </c>
       <c r="G4" t="s">
-        <v>74</v>
+        <v>89</v>
       </c>
     </row>
     <row r="5" spans="1:7">
       <c r="A5" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B5" t="s">
-        <v>60</v>
+        <v>75</v>
       </c>
       <c r="C5" t="s">
-        <v>63</v>
+        <v>78</v>
       </c>
       <c r="D5" t="s">
-        <v>67</v>
+        <v>82</v>
       </c>
       <c r="E5" t="s">
-        <v>71</v>
+        <v>86</v>
       </c>
       <c r="F5">
         <f> ,435</f>
         <v>0</v>
       </c>
       <c r="G5" t="s">
-        <v>74</v>
+        <v>89</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:F8"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:6">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>90</v>
+      </c>
+      <c r="D1" t="s">
+        <v>91</v>
+      </c>
+      <c r="E1" t="s">
+        <v>25</v>
+      </c>
+      <c r="F1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
+      <c r="A2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C2" t="s">
+        <v>92</v>
+      </c>
+      <c r="D2" t="s">
+        <v>96</v>
+      </c>
+      <c r="E2" t="s">
+        <v>101</v>
+      </c>
+      <c r="F2" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6">
+      <c r="A3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" t="s">
+        <v>93</v>
+      </c>
+      <c r="D3" t="s">
+        <v>97</v>
+      </c>
+      <c r="E3" t="s">
+        <v>29</v>
+      </c>
+      <c r="F3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6">
+      <c r="A4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" t="s">
+        <v>94</v>
+      </c>
+      <c r="D4" t="s">
+        <v>94</v>
+      </c>
+      <c r="E4" t="s">
+        <v>94</v>
+      </c>
+      <c r="F4" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6">
+      <c r="A5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" t="s">
+        <v>94</v>
+      </c>
+      <c r="D5" t="s">
+        <v>94</v>
+      </c>
+      <c r="E5" t="s">
+        <v>94</v>
+      </c>
+      <c r="F5" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6">
+      <c r="A6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C6" t="s">
+        <v>92</v>
+      </c>
+      <c r="D6" t="s">
+        <v>98</v>
+      </c>
+      <c r="E6" t="s">
+        <v>30</v>
+      </c>
+      <c r="F6" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6">
+      <c r="A7" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7" t="s">
+        <v>12</v>
+      </c>
+      <c r="C7" t="s">
+        <v>92</v>
+      </c>
+      <c r="D7" t="s">
+        <v>99</v>
+      </c>
+      <c r="E7" t="s">
+        <v>31</v>
+      </c>
+      <c r="F7" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6">
+      <c r="A8" t="s">
+        <v>11</v>
+      </c>
+      <c r="B8" t="s">
+        <v>12</v>
+      </c>
+      <c r="C8" t="s">
+        <v>95</v>
+      </c>
+      <c r="D8" t="s">
+        <v>100</v>
+      </c>
+      <c r="E8" t="s">
+        <v>32</v>
+      </c>
+      <c r="F8" t="s">
+        <v>35</v>
       </c>
     </row>
   </sheetData>

</xml_diff>